<commit_message>
Cap nhat he thong danh gia xep loai vien chuc CBQL GV NV
</commit_message>
<xml_diff>
--- a/public/downloads/Import công việc.xlsx
+++ b/public/downloads/Import công việc.xlsx
@@ -524,13 +524,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="3"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" style="7" min="4" max="5"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="11"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -621,17 +621,17 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng và ban hành Kế hoạch giáo dục nhà trường, kế hoạch phát triển chiến lược năm học 2026 - 2027</t>
+          <t>Tổng hợp kết quả đánh giá, xếp loại chất lượng viên chức, người lao động cuối năm học 2025 - 2026 theo Nghị định 90/2020 &amp; 48/2023</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
@@ -645,7 +645,7 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch số 01/KH-THPT; Nghị quyết Hội đồng trường</t>
+          <t>Biên bản họp Hội đồng đánh giá xếp loại viên chức năm học 2025-2026</t>
         </is>
       </c>
     </row>
@@ -655,17 +655,17 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Phê duyệt kế hoạch giáo dục của các tổ chuyên môn, tổ văn phòng và các tổ chức đoàn thể trong nhà trường</t>
+          <t>Ban hành Quyết định công nhận kết quả đánh giá, xếp loại viên chức, người lao động và công khai toàn trường</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
@@ -679,27 +679,27 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch năm học các tổ TN, XH, VP, Công đoàn, Đoàn TN</t>
+          <t>Quyết định số 85/QĐ-THPT công nhận kết quả xếp loại</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo tổ chức Hội nghị cán bộ, viên chức, người lao động năm học 2026 - 2027</t>
+          <t>Chỉ đạo thẩm định hồ sơ thi đua, sáng kiến kinh nghiệm của CBGVNV đề nghị công nhận LĐTT, CSTĐ cơ sở năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
@@ -713,27 +713,27 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Nghị quyết Hội nghị CBVC-NLĐ năm học 2026-2027</t>
+          <t>Biên bản thẩm định hồ sơ sáng kiến kinh nghiệm và thi đua</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng lịch công tác tuần, tháng, quý và chương trình điều hành tổng thể hoạt động sư phạm nhà trường</t>
+          <t>Tổ chức họp Hội đồng Thi đua - Khen thưởng nhà trường xét duyệt danh hiệu và hoàn thiện tờ trình nộp Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
+          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
@@ -747,27 +747,27 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Lịch công tác tuần đưa lên website và bảng tin điện tử</t>
+          <t>Tờ trình số 28/TTr-THPT đề nghị khen thưởng năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Phân công nhiệm vụ cụ thể cho các Phó Hiệu trưởng, Tổ trưởng chuyên môn và các bộ phận phụ trách</t>
+          <t>Rà soát, chuẩn bị đầy đủ phòng thi, camera giám sát, thiết bị PCCC, phòng bảo quản đề thi, bài thi phục vụ Điểm thi tốt nghiệp THPT năm 2026</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
+          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
@@ -781,27 +781,27 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Quyết định phân công nhiệm vụ cán bộ quản lý năm học</t>
+          <t>Biên bản kiểm tra điều kiện CSVC Điểm thi tốt nghiệp THPT năm 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức họp giao ban Ban Giám hiệu và họp Hội đồng sư phạm định kỳ hàng tháng</t>
+          <t>Phối hợp với chính quyền địa phương, công an, y tế bảo đảm an ninh trật tự, an toàn giao thông và phòng chống dịch bệnh kỳ thi tốt nghiệp</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
@@ -815,27 +815,27 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp Hội đồng sư phạm từ tháng 9/2026 đến 5/2027</t>
+          <t>Kế hoạch phối hợp liên ngành bảo đảm an ninh trật tự kỳ thi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo, đôn đốc và đánh giá xếp loại thi đua cán bộ, giáo viên, nhân viên hàng tháng</t>
+          <t>Thành lập Hội đồng tuyển sinh lớp 10 THPT năm học 2026 - 2027; ban hành Thông báo hướng dẫn tuyển sinh</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
@@ -849,27 +849,27 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Bảng tổng hợp xếp loại thi đua tháng các tổ</t>
+          <t>Quyết định thành lập HĐTS và Thông báo số 12/TB-THPT tuyển sinh lớp 10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra, đôn đốc tiến độ thực hiện chương trình giảng dạy và quy chế chuyên môn toàn trường</t>
+          <t>Chỉ đạo thu nhận hồ sơ, xét tuyển, hoàn thành duyệt danh sách trúng tuyển lớp 10 trình Sở GD&amp;ĐT phê duyệt</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="E16" s="9" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Hồ sơ theo dõi tiến độ chương trình trên hệ thống VnEdu</t>
+          <t>Danh sách học sinh trúng tuyển lớp 10 đã được Sở GD&amp;ĐT phê duyệt</t>
         </is>
       </c>
     </row>
@@ -893,17 +893,17 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Bộ tiêu chí và quy định đánh giá, xếp loại viên chức, người lao động năm học 2026 - 2027</t>
+          <t>Xây dựng Kế hoạch bồi dưỡng chính trị hè năm 2026 và bồi dưỡng chuyên môn nghiệp vụ cho cán bộ quản lý, giáo viên</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
@@ -917,27 +917,27 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>Quy định số 02/QĐ-THPT về tiêu chí thi đua xếp loại</t>
+          <t>Kế hoạch số 45/KH-THPT bồi dưỡng chính trị và chuyên môn hè 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Thành lập Hội đồng đánh giá, phân loại chất lượng viên chức và người lao động nhà trường</t>
+          <t>Chỉ đạo rà soát, xét duyệt quyết toán thu chi ngân sách 6 tháng đầu năm 2026 và đối chiếu kho bạc</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
+          <t>N2_1158 - Xét duyệt quyết toán ngân sách Nhà nước hàng năm</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>15/05/2027</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="E18" s="9" t="n">
@@ -951,27 +951,27 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Quyết định thành lập Hội đồng ĐGXL viên chức</t>
+          <t>Báo cáo quyết toán tài chính ngân sách 6 tháng đầu năm 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức đánh giá, tổng hợp kết quả và ban hành quyết định công nhận xếp loại viên chức cuối năm</t>
+          <t>Cử cán bộ quản lý, giáo viên tham gia đầy đủ các lớp tập huấn SGK, phương pháp giảng dạy và ứng dụng AI do Sở GD&amp;ĐT tổ chức</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp xét thi đua và Thông báo kết quả ĐGXL</t>
+          <t>Quyết định cử cán bộ, giáo viên dự tập huấn hè năm 2026</t>
         </is>
       </c>
     </row>
@@ -995,17 +995,17 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng và triển khai Kế hoạch kiểm tra nội bộ trường học năm học 2026 - 2027 (toàn diện &amp; chuyên đề)</t>
+          <t>Kiểm tra, nghiệm thu công tác sửa chữa phòng học, bàn ghế, hệ thống điện nước, mái che và vệ sinh khuôn viên trường trong hè</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>N2_1042 - Tham mưu công tác kiểm tra các kỳ thi, kiểm tra chuyên môn</t>
+          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E20" s="9" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch số 03/KH-KTNB và các biên bản kiểm tra chuyên đề</t>
+          <t>Biên bản nghiệm thu tu sửa cơ sở vật chất hè 2026</t>
         </is>
       </c>
     </row>
@@ -1029,17 +1029,17 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra hồ sơ chuyên môn, giáo án điện tử, sổ điểm và nền nếp dạy học của giáo viên</t>
+          <t>Rà soát, mua sắm bổ sung thiết bị dạy học tối thiểu, sách thư viện và hóa chất thí nghiệm chuẩn bị năm học mới 2026 - 2027</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>N2_1042 - Tham mưu công tác kiểm tra các kỳ thi, kiểm tra chuyên môn</t>
+          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
@@ -1053,27 +1053,27 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm tra hồ sơ giáo viên định kỳ 2 lần/học kỳ</t>
+          <t>Hợp đồng mua sắm thiết bị dạy học và sách thư viện</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo và giám sát công tác tổ chức kiểm tra định kỳ (giữa kỳ, cuối kỳ) và thi thử tốt nghiệp THPT</t>
+          <t>Ban hành Quyết định phân công nhiệm vụ cán bộ quản lý, phân công chuyên môn giáo viên và biên chế học sinh các lớp năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>N2_1042 - Tham mưu công tác kiểm tra các kỳ thi, kiểm tra chuyên môn</t>
+          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>20/08/2026</t>
         </is>
       </c>
       <c r="E22" s="9" t="n">
@@ -1087,27 +1087,27 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch kiểm tra định kỳ và biên bản giám sát coi, chấm thi</t>
+          <t>Quyết định số 102/QĐ-THPT về phân công nhiệm vụ năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch ôn tập tốt nghiệp THPT năm 2027 cho học sinh khối 12; phân công GV cốt cán phụ trách</t>
+          <t>Chỉ đạo tổ chức ngày tựu trường, đón học sinh lớp 10 và tổ chức tuần sinh hoạt tập thể đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>N3_661 - Ban hành Kế hoạch tổ chức kỳ thi tốt nghiệp THPT năm 2026 của Sở GDĐT</t>
+          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>15/11/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
@@ -1121,27 +1121,27 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch ôn tập tốt nghiệp THPT năm học 2026-2027</t>
+          <t>Kế hoạch tựu trường và tuần sinh hoạt tập thể học sinh đầu năm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức các đợt thi thử tốt nghiệp THPT, phân tích phổ điểm để chỉ đạo đổi mới phương pháp dạy ôn</t>
+          <t>Xây dựng Kế hoạch và chỉ đạo tổ chức Lễ Khai giảng năm học mới 2026 - 2027 trang trọng, ý nghĩa, an toàn và tiết kiệm</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>N3_661 - Ban hành Kế hoạch tổ chức kỳ thi tốt nghiệp THPT năm 2026 của Sở GDĐT</t>
+          <t>N3_666 - Kế hoạch tham dự Lễ Khai giảng năm học 2026 - 2027 tại các cơ sở giáo dục trên địa bàn tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>20/05/2027</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E24" s="9" t="n">
@@ -1155,27 +1155,27 @@
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo phân tích phổ điểm các đợt thi khảo sát khối 12</t>
+          <t>Kế hoạch tổ chức Lễ Khai giảng năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Chuẩn bị đầy đủ các điều kiện cơ sở vật chất, an ninh trật tự phục vụ Điểm thi tốt nghiệp THPT</t>
+          <t>Xây dựng và ban hành Kế hoạch giáo dục nhà trường, kế hoạch thực hiện nhiệm vụ trọng tâm năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>N3_661 - Ban hành Kế hoạch tổ chức kỳ thi tốt nghiệp THPT năm 2026 của Sở GDĐT</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>20/06/2027</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
@@ -1189,27 +1189,27 @@
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm tra cơ sở vật chất Điểm thi tốt nghiệp</t>
+          <t>Kế hoạch giáo dục nhà trường năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo xây dựng dự toán ngân sách Nhà nước và Quy chế chi tiêu nội bộ năm học 2026 - 2027</t>
+          <t>Phê duyệt kế hoạch giáo dục của các tổ chuyên môn, tổ văn phòng và các bộ phận trong nhà trường năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>N2_1150 - Xây dựng dự toán ngân sách Nhà nước hàng năm</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="E26" s="9" t="n">
@@ -1223,27 +1223,27 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Dự toán ngân sách năm 2027 và Quy chế chi tiêu nội bộ sửa đổi</t>
+          <t>Kế hoạch năm học các tổ TN, XH, VP đã phê duyệt</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Quản lý, sử dụng nguồn tài chính ngân sách đúng quy định, công khai minh bạch tài chính trường học</t>
+          <t>Chỉ đạo tổ chức thành công Hội nghị cán bộ, viên chức, người lao động năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>N2_1150 - Xây dựng dự toán ngân sách Nhà nước hàng năm</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo công khai tài chính định kỳ quý, năm theo Thông tư</t>
+          <t>Nghị quyết Hội nghị CBVC-NLĐ năm học 2026-2027</t>
         </is>
       </c>
     </row>
@@ -1267,12 +1267,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Rà soát, mua sắm bổ sung, sửa chữa cơ sở vật chất, thiết bị dạy học phục vụ năm học mới 2026 - 2027</t>
+          <t>Xây dựng lịch công tác tuần, tháng 9 và chương trình điều hành tổng thể hoạt động sư phạm toàn trường</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
+          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -1291,27 +1291,27 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm kê và danh mục mua sắm sửa chữa tài sản</t>
+          <t>Lịch công tác tuần tháng 9/2026 đăng tải trên cổng thông tin điện tử</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo công tác bảo đảm an toàn trường học, phòng chống cháy nổ, vệ sinh môi trường xanh - sạch - đẹp</t>
+          <t>Tổ chức họp giao ban BGH và họp Hội đồng sư phạm tháng 9/2026 đánh giá triển khai nhiệm vụ năm học mới</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
@@ -1325,27 +1325,27 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch an toàn trường học và biên bản tự kiểm tra PCCC</t>
+          <t>Biên bản họp Hội đồng sư phạm tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Thông báo Lịch tiếp công dân của Hiệu trưởng, bố trí phòng tiếp dân và mở sổ theo dõi tiếp dân</t>
+          <t>Kiểm tra, đôn đốc tiến độ thực hiện chương trình giảng dạy và nền nếp chuyên môn tháng 9</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
@@ -1359,27 +1359,27 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>Thông báo lịch tiếp công dân năm học 2026-2027</t>
+          <t>Báo cáo kiểm tra nền nếp dạy học tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện tiếp công dân định kỳ và đột xuất; xử lý, giải quyết kịp thời đơn thư khiếu nại, phản ánh</t>
+          <t>Tổng hợp số liệu đầu năm, kiểm tra việc ổn định nền nếp dạy học tháng 9 và báo cáo Sở GD&amp;ĐT đúng thời hạn</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
+          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="E31" s="9" t="n">
@@ -1393,27 +1393,27 @@
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi tiếp công dân và giải quyết khiếu nại kiến nghị</t>
+          <t>Báo cáo tình hình triển khai nhiệm vụ đầu năm học gửi Sở GD&amp;ĐT</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo triển khai mạnh mẽ ứng dụng CNTT, phần mềm quản lý trường học VnEdu, học bạ số và chữ ký số</t>
+          <t>Chỉ đạo triển khai công tác tuyên truyền phổ biến pháp luật, an toàn giao thông và cam kết an ninh trật tự trường học tháng 9</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>N2_1107 - Báo cáo tổng kết đánh giá tình hình triển khai nhiệm vụ ứng dụng công nghệ thông tin và chuyển đổi số</t>
+          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
@@ -1427,27 +1427,27 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>Hồ sơ triển khai 100% học bạ số và chữ ký số giáo viên</t>
+          <t>Bản cam kết an toàn giao thông và phòng chống bạo lực học đường</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng báo cáo tổng kết chuyển đổi số và phát triển kho học liệu điện tử phục vụ giáo viên, học sinh</t>
+          <t>Ban hành Thông báo Lịch tiếp công dân năm học 2026 - 2027; tiếp nhận và giải quyết kịp thời phản ánh của phụ huynh đầu năm học</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>N2_1107 - Báo cáo tổng kết đánh giá tình hình triển khai nhiệm vụ ứng dụng công nghệ thông tin và chuyển đổi số</t>
+          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo chuyển đổi số ngành giáo dục năm học 2026-2027</t>
+          <t>Thông báo lịch tiếp công dân năm học 2026-2027 và sổ tiếp dân</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Soạn Kế hoạch bài dạy (giáo án) đúng chuẩn Công văn 5512/BGDĐT, tích hợp năng lực số và ứng dụng AI</t>
+          <t>Hoàn thành chấm bài, vào điểm, tổng kết đánh giá xếp loại học sinh cuối năm học 2025 - 2026 trên phần mềm VnEdu</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>Giáo án điện tử môn giảng dạy lưu trên hệ thống CSDL trường</t>
+          <t>Sổ điểm điện tử năm học 2025-2026 trên hệ thống VnEdu</t>
         </is>
       </c>
     </row>
@@ -1505,17 +1505,17 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch dạy học môn học cá nhân và kế hoạch kiểm tra đánh giá định kỳ theo phân phối chương trình</t>
+          <t>Thực hiện nhiệm vụ coi thi, chấm thi kỳ thi tuyển sinh lớp 10 THPT và kỳ thi tốt nghiệp THPT năm 2026 theo điều động của Sở</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
@@ -1529,27 +1529,27 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>KHDH cá nhân đã được Tổ trưởng và BGH phê duyệt</t>
+          <t>Quyết định điều động cán bộ coi thi, chấm thi của Sở GD&amp;ĐT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế học liệu số, bài giảng điện tử tương tác và ngân hàng câu hỏi trắc nghiệm rèn luyện trực tuyến</t>
+          <t>Hoàn thiện hồ sơ sáng kiến kinh nghiệm, hồ sơ minh chứng đề nghị đánh giá xếp loại viên chức cuối năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Kho bài giảng điện tử và link học liệu số trên cổng web trường</t>
+          <t>Báo cáo sáng kiến kinh nghiệm và phiếu tự đánh giá viên chức</t>
         </is>
       </c>
     </row>
@@ -1573,17 +1573,17 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện đầy đủ, nghiêm túc số tiết dạy theo phân công thời khóa biểu; lên lớp đúng giờ, không bỏ tiết</t>
+          <t>Tham gia đầy đủ lớp bồi dưỡng chính trị hè năm 2026 và hoàn thành bài thu hoạch đạt yêu cầu</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>Sổ đầu bài các lớp, sổ theo dõi chuyên môn của tổ</t>
+          <t>Bài thu hoạch bồi dưỡng chính trị hè 2026</t>
         </is>
       </c>
     </row>
@@ -1607,17 +1607,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Tích cực đổi mới phương pháp dạy học, phát huy tính tích cực, chủ động, sáng tạo và năng lực tự học của học sinh</t>
+          <t>Hoàn thành khóa tập huấn chuyên môn, bồi dưỡng SGK và đổi mới phương pháp dạy học theo CT GDPT 2018 trong hè</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E38" s="9" t="n">
@@ -1631,27 +1631,27 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>Phiếu đánh giá tiết dạy đạt loại Khá, Giỏi</t>
+          <t>Giấy chứng nhận / kết quả hoàn thành tập huấn bồi dưỡng hè 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Tham gia đầy đủ các buổi sinh hoạt chuyên môn của tổ theo định hướng nghiên cứu bài học (tối thiểu 2 lần/tháng)</t>
+          <t>Xây dựng Kế hoạch dạy học môn học cá nhân năm học 2026 - 2027 nộp Tổ trưởng chuyên môn phê duyệt</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E39" s="9" t="n">
@@ -1665,27 +1665,27 @@
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>Biên bản sinh hoạt tổ chuyên môn</t>
+          <t>Kế hoạch dạy học cá nhân năm học 2026-2027 có xác nhận của Tổ trưởng</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện dự giờ đồng nghiệp đúng quy định (đạt 18-20 tiết/năm), trao đổi, rút kinh nghiệm chuyên môn</t>
+          <t>Nhận lớp chủ nhiệm, tổ chức cho học sinh tựu trường, ổn định tổ chức lớp và phổ biến nội quy học sinh</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="E40" s="9" t="n">
@@ -1699,27 +1699,27 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>Sổ dự giờ của giáo viên có đầy đủ nhận xét, xếp loại</t>
+          <t>Biên bản họp lớp đầu năm và danh sách ban cán sự lớp</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng ma trận, bản đặc tả và đề kiểm tra định kỳ (giữa kỳ, cuối kỳ) theo đúng định hướng đánh giá năng lực</t>
+          <t>Chuẩn bị trang phục, hướng dẫn học sinh tham gia Lễ Khai giảng năm học 2026 - 2027 trang nghiêm, đầy đủ quân số</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
@@ -1733,27 +1733,27 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>Hồ sơ ngân hàng đề kiểm tra nộp tổ chuyên môn</t>
+          <t>Sổ chủ nhiệm ghi nhận quân số dự Khai giảng 100%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Chấm bài kiểm tra chính xác, trả bài kịp thời; cập nhật điểm số thường xuyên và định kỳ đầy đủ lên VnEdu</t>
+          <t>Tổ chức Hội nghị Ban đại diện Cha mẹ học sinh lớp đầu năm học 2026 - 2027; lập biên bản họp đúng quy định</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
@@ -1767,27 +1767,27 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Sổ điểm điện tử trên VnEdu đúng tiến độ theo từng mốc thời gian</t>
+          <t>Biên bản họp phụ huynh học sinh đầu năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Tham gia công tác coi thi, chấm thi kiểm tra định kỳ, thi thử tốt nghiệp THPT an toàn, nghiêm túc, đúng quy chế</t>
+          <t>Cập nhật hồ sơ học sinh, hoàn thiện cơ sở dữ liệu lý lịch và thông tin liên lạc của học sinh trên hệ thống VnEdu</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
@@ -1801,27 +1801,27 @@
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>Bảng tổng hợp điểm chấm thi và biên bản coi thi</t>
+          <t>Dữ liệu hồ sơ học sinh lớp chủ nhiệm trên hệ thống CSDL trường</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Phát hiện, lập danh sách và trực tiếp tham gia bồi dưỡng đội tuyển học sinh giỏi môn phụ trách thi cấp trường, cấp tỉnh</t>
+          <t>Soạn Kế hoạch bài dạy (giáo án) các tuần học tháng 9/2026 đúng chuẩn Công văn 5512/BGDĐT, tích hợp năng lực số và AI</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>30/03/2027</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E44" s="9" t="n">
@@ -1835,27 +1835,27 @@
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch bồi dưỡng HSG và kết quả thi HSG cấp tỉnh</t>
+          <t>Giáo án các tuần 1, 2, 3, 4 tháng 9 lưu trên hệ thống CSDL giáo án</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng kế hoạch và tổ chức dạy phụ đạo, giúp đỡ học sinh học lực yếu kém, có nguy cơ không đạt chuẩn</t>
+          <t>Thiết kế bài giảng điện tử và học liệu số tương tác phục vụ dạy học các chuyên đề đầu năm học mới</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>20/05/2027</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch phụ đạo học sinh yếu kém và theo dõi sự tiến bộ</t>
+          <t>Link bài giảng điện tử và học liệu số tải lên thư viện trường</t>
         </is>
       </c>
     </row>
@@ -1879,17 +1879,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Viết sáng kiến kinh nghiệm hoặc giải pháp đổi mới giáo dục được Hội đồng chuyên môn nhà trường nghiệm thu đạt loại Khá trở lên</t>
+          <t>Thực hiện nghiêm túc thời khóa biểu tháng 9/2026, lên lớp đúng giờ, duy trì tốt nền nếp và kỷ luật dạy học</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>15/04/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E46" s="9" t="n">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>Văn bản báo cáo sáng kiến kinh nghiệm năm học 2026-2027</t>
+          <t>Sổ đầu bài các lớp giảng dạy tháng 9/2026</t>
         </is>
       </c>
     </row>
@@ -1913,17 +1913,17 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Hướng dẫn học sinh tham gia Cuộc thi Khoa học kỹ thuật (KHKT) cấp trường/cấp tỉnh hoặc các cuộc thi trí tuệ</t>
+          <t>Tham gia các buổi sinh hoạt tổ chuyên môn đầu năm học: thống nhất ma trận đề, kế hoạch giáo dục và quy chế tổ</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>15/01/2027</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
@@ -1937,27 +1937,27 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Dự án dự thi KHKT học sinh và Quyết định công nhận</t>
+          <t>Biên bản họp tổ chuyên môn tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng kế hoạch chủ nhiệm lớp, nắm vững hoàn cảnh từng học sinh; duy trì sĩ số lớp 100%, phòng chống bỏ học</t>
+          <t>Thực hiện dự giờ đồng nghiệp tháng 9 theo kế hoạch tổ chuyên môn (đạt 2 tiết/tháng), trao đổi kinh nghiệm sư phạm</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="E48" s="9" t="n">
@@ -1971,27 +1971,27 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>Sổ công tác chủ nhiệm lớp, biên bản thăm gia đình học sinh</t>
+          <t>Sổ dự giờ giáo viên có nhận xét và đánh giá tiết dạy</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức sinh hoạt lớp, giáo dục đạo đức, kỹ năng sống, văn hóa ứng xử học đường và phòng chống bạo lực học đường</t>
+          <t>Thực hiện kiểm tra đánh giá thường xuyên học sinh theo đúng kế hoạch; chấm bài và vào điểm VnEdu kịp thời</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
@@ -2005,27 +2005,27 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>Giáo án tiết sinh hoạt lớp theo chủ đề hàng tuần</t>
+          <t>Điểm kiểm tra thường xuyên tháng 9 cập nhật trên VnEdu</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức các buổi họp phụ huynh học sinh đầu năm, giữa kỳ, cuối năm; giữ mối liên lạc chặt chẽ với cha mẹ học sinh qua Zalo/Smas</t>
+          <t>Khảo sát chất lượng đầu năm, phát hiện và lập danh sách học sinh năng khiếu để bồi dưỡng đội tuyển HSG môn phụ trách</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E50" s="9" t="n">
@@ -2039,27 +2039,27 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp Ban đại diện cha mẹ học sinh lớp</t>
+          <t>Danh sách đội tuyển HSG và Kế hoạch bồi dưỡng HSG</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Đánh giá, nhận xét rèn luyện và học tập của học sinh; cập nhật kết quả hạnh kiểm, khen thưởng đầy đủ lên phần mềm CSDL</t>
+          <t>Lập danh sách học sinh học lực yếu kém đầu năm học để xây dựng phương án dạy phụ đạo, kèm cặp nâng cao chất lượng</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E51" s="9" t="n">
@@ -2073,27 +2073,27 @@
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Hồ sơ đánh giá rèn luyện học kỳ 1, học kỳ 2 trên VnEdu</t>
+          <t>Kế hoạch phụ đạo học sinh có kết quả khảo sát đầu năm thấp</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Tham gia đầy đủ các lớp bồi dưỡng thường xuyên, bồi dưỡng chuyên môn nghiệp vụ theo quy định của Sở GD&amp;ĐT</t>
+          <t>Đăng ký tên đề tài Sáng kiến kinh nghiệm hoặc Đề tài nghiên cứu khoa học sư phạm ứng dụng năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E52" s="9" t="n">
@@ -2107,17 +2107,17 @@
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Giấy chứng nhận bồi dưỡng thường xuyên hoặc kết quả trên cổng bồi dưỡng</t>
+          <t>Phiếu đăng ký đề tài SKKN năm học 2026-2027 nộp Tổ chuyên môn</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Tự bồi dưỡng nâng cao trình độ chuyên môn, năng lực ứng dụng CNTT, ngoại ngữ và kỹ năng sư phạm hiện đại</t>
+          <t>Xây dựng Kế hoạch tự bồi dưỡng thường xuyên cá nhân năm học 2026 - 2027 theo quy định của Bộ và Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E53" s="9" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch tự học và bài thu hoạch bồi dưỡng thường xuyên cá nhân</t>
+          <t>Bản kế hoạch tự học, bồi dưỡng thường xuyên năm học 2026-2027</t>
         </is>
       </c>
     </row>
@@ -2151,17 +2151,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Tiếp nhận, kiểm tra tính hợp pháp, hợp lệ của chứng từ thu chi, đề nghị thanh toán theo Quy chế chi tiêu nội bộ</t>
+          <t>Rút dự toán thanh toán tiền lương, các khoản phụ cấp tháng 6/2026 cho cán bộ, giáo viên, nhân viên đúng thời hạn</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>N1_594 - Thu thập và xử lý thông tin số liệu chứng từ kế toán</t>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="E54" s="9" t="n">
@@ -2175,27 +2175,27 @@
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>Bộ chứng từ thanh toán thu - chi lưu tại phòng Tài chính - Kế toán</t>
+          <t>Giấy rút dự toán ngân sách và bảng thanh toán lương tháng 6/2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Lập phiếu thu, phiếu chi, giấy đề nghị rút hạn mức, ủy nhiệm chi và cập nhật số liệu chính xác vào phần mềm MISA</t>
+          <t>Tiếp nhận, đăng ký, chuyển giao kịp thời văn bản chỉ đạo của Sở về thi tốt nghiệp THPT và tuyển sinh lớp 10 năm 2026</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>N1_594 - Thu thập và xử lý thông tin số liệu chứng từ kế toán</t>
+          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="E55" s="9" t="n">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>Dữ liệu kế toán xuất từ phần mềm MISA</t>
+          <t>Sổ theo dõi văn bản đến tháng 6/2026 trên iOffice</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Lập hồ sơ rút dự toán thanh toán tiền lương, các khoản phụ cấp, chế độ bảo hiểm xã hội, BHYT, KPCĐ đúng hạn hàng tháng</t>
+          <t>Chuẩn bị cơ số thuốc, vật tư y tế, phòng y tế phục vụ Điểm thi tốt nghiệp THPT năm 2026 tại trường an toàn</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="E56" s="9" t="n">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>Bảng thanh toán tiền lương có chữ ký và xác nhận của KBNN</t>
+          <t>Biên bản kiểm tra điều kiện y tế phục vụ kỳ thi tốt nghiệp 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Đối chiếu số liệu tài khoản tiền gửi, tiền dự toán ngân sách định kỳ hàng tháng, quý với Kho bạc Nhà nước</t>
+          <t>Bảo dưỡng, kiểm tra hệ thống máy vi tính, đường truyền internet, camera giám sát phục vụ thi tốt nghiệp THPT 2026</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="E57" s="9" t="n">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>Biên bản xác nhận số dư tài khoản tại Kho bạc Nhà nước</t>
+          <t>Nhật ký kiểm tra thiết bị CNTT phục vụ kỳ thi</t>
         </is>
       </c>
     </row>
@@ -2287,17 +2287,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Lập báo cáo quyết toán tài chính ngân sách năm học và quyết toán ngân sách nhà nước năm đúng hạn</t>
+          <t>Thu hồi SGK, tài liệu tham khảo cho mượn năm học 2025 - 2026; xử lý kỹ thuật và sắp xếp lại kho sách thư viện</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>31/01/2027</t>
+          <t>28/06/2026</t>
         </is>
       </c>
       <c r="E58" s="9" t="n">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo tài chính năm 2026 gửi Sở GD&amp;ĐT và Kho bạc</t>
+          <t>Sổ theo dõi mượn trả sách thư viện cuối năm</t>
         </is>
       </c>
     </row>
@@ -2321,17 +2321,17 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện công khai tài chính quý, năm và phục vụ chu đáo các đợt thanh tra, kiểm tra, kiểm toán tài chính</t>
+          <t>Thực hiện đối chiếu số dư tài khoản tiền gửi và hạn mức kinh phí 6 tháng đầu năm 2026 với Kho bạc Nhà nước</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="E59" s="9" t="n">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>Biểu mẫu công khai tài chính niêm yết tại bảng tin cơ quan</t>
+          <t>Biên bản đối chiếu tài khoản với KBNN kỳ 6 tháng đầu năm 2026</t>
         </is>
       </c>
     </row>
@@ -2355,17 +2355,17 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Tiếp nhận, đăng ký, chuyển giao kịp thời văn bản đến trên hệ thống quản lý văn bản iOffice/VNPT iOffice</t>
+          <t>Lập báo cáo tài chính và báo cáo quyết toán ngân sách nhà nước 6 tháng đầu năm 2026 nộp Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="E60" s="9" t="n">
@@ -2379,27 +2379,27 @@
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi văn bản đến và dữ liệu trên phần mềm quản lý văn bản</t>
+          <t>Báo cáo quyết toán ngân sách 6 tháng đầu năm 2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra thể thức, lấy số, phát hành văn bản đi của nhà trường đảm bảo đúng quy chuẩn kỹ thuật văn bản</t>
+          <t>Tiếp nhận hồ sơ, sao lục học bạ và cấp phát giấy chứng nhận tốt nghiệp tạm thời cho học sinh khối 12 năm 2026</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="E61" s="9" t="n">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>Sổ văn bản đi năm học 2026-2027</t>
+          <t>Sổ cấp phát văn bằng chứng chỉ, giấy chứng nhận tốt nghiệp tạm thời</t>
         </is>
       </c>
     </row>
@@ -2423,17 +2423,17 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Quản lý và sử dụng con dấu, USB token chữ ký số cơ quan an toàn, chặt chẽ, đúng thẩm quyền</t>
+          <t>Thu thập, phân loại và lưu trữ toàn bộ hồ sơ thi tốt nghiệp THPT 2026, hồ sơ tuyển sinh 10 và hồ sơ thi đua năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+          <t>N1_604 - Thu thập hồ sơ tài liệu vào kho lưu trữ, phục vụ khai thác, sử dụng tài liệu lưu trữ</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E62" s="9" t="n">
@@ -2447,27 +2447,27 @@
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi đóng dấu và nhật ký ký số điện tử</t>
+          <t>Mục lục hồ sơ tài liệu nộp lưu trữ cơ quan đợt hè 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện tiếp nhận và giải quyết thủ tục hành chính: cấp bản sao học bạ, giấy chứng nhận tốt nghiệp cho học sinh đúng hạn</t>
+          <t>Chi trả kịp thời tiền làm nhiệm vụ coi thi, chấm thi và tiền phụ cấp làm việc hè cho cán bộ, giáo viên đúng danh sách</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="E63" s="9" t="n">
@@ -2481,27 +2481,27 @@
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>Sổ cấp phát văn bằng chứng chỉ, giấy chứng nhận</t>
+          <t>Bảng thanh toán tiền làm nhiệm vụ thi có chữ ký người nhận</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Thu thập, phân loại, chỉnh lý hồ sơ thi đua, bài thi tốt nghiệp, sổ điểm của các năm học đưa vào kho lưu trữ</t>
+          <t>Lập dự toán kinh phí mua sắm, sửa chữa cơ sở vật chất, bàn ghế phục vụ khai giảng và năm học mới 2026 - 2027</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>N1_604 - Thu thập hồ sơ tài liệu vào kho lưu trữ, phục vụ khai thác, sử dụng tài liệu lưu trữ</t>
+          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E64" s="9" t="n">
@@ -2515,27 +2515,27 @@
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>Danh mục hồ sơ tài liệu nộp lưu trữ cơ quan năm học</t>
+          <t>Dự toán chi tiết mua sắm, sửa chữa CSVC đầu năm học mới</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Bảo quản an toàn kho tài liệu lưu trữ, chống ẩm, mối mọt; phục vụ tra cứu hồ sơ nhanh chóng, chính xác</t>
+          <t>Kiểm kê, vệ sinh, bảo dưỡng toàn bộ thiết bị dạy học, hóa chất, phòng thực hành Lý, Hóa, Sinh trong dịp hè</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>N1_604 - Thu thập hồ sơ tài liệu vào kho lưu trữ, phục vụ khai thác, sử dụng tài liệu lưu trữ</t>
+          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E65" s="9" t="n">
@@ -2549,27 +2549,27 @@
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>Nhật ký khai thác, sử dụng tài liệu lưu trữ</t>
+          <t>Biên bản kiểm kê thiết bị dạy học và phòng bộ môn hè 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Quản lý quỹ tiền mặt tuyệt đối an toàn; thực hiện thu - chi tiền mặt chính xác, kịp thời theo lệnh thu - chi hợp lệ</t>
+          <t>Tiếp nhận, đóng dấu nghiệp vụ và cấp phát SGK mới, tài liệu hướng dẫn giảng dạy cho GV và HS chuẩn bị năm học mới</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E66" s="9" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
-          <t>Sổ quỹ tiền mặt có đối chiếu hàng ngày giữa Thủ quỹ và Kế toán</t>
+          <t>Sổ đăng ký cá biệt và danh sách cấp phát sách giáo khoa mới</t>
         </is>
       </c>
     </row>
@@ -2593,17 +2593,17 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Chi trả kịp thời tiền học bổng, tiền hỗ trợ chi phí học tập cho học sinh diện chính sách, vùng cao đầy đủ chữ ký</t>
+          <t>Bảo dưỡng phòng máy tính tin học, kiểm tra tài khoản VnEdu, CSDL ngành, học bạ số và chữ ký số chuẩn bị năm học mới</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E67" s="9" t="n">
@@ -2617,27 +2617,27 @@
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>Danh sách học sinh nhận tiền chính sách có chữ ký người nhận</t>
+          <t>Biên bản kiểm tra hệ thống CNTT và phần mềm quản lý trường học</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Lập kế hoạch quản lý, bảo dưỡng và chuẩn bị thiết bị, hóa chất phục vụ các tiết dạy thực hành môn Lý, Hóa, Sinh</t>
+          <t>Lập hồ sơ rút dự toán thanh toán tiền lương, phụ cấp tháng 9/2026 và trích nộp BHXH, BHYT, KPCĐ đúng thời hạn</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="E68" s="9" t="n">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Sổ mượn trả thiết bị và nhật ký sử dụng phòng thí nghiệm</t>
+          <t>Bảng thanh toán lương tháng 9/2026 và chứng từ nộp bảo hiểm xã hội</t>
         </is>
       </c>
     </row>
@@ -2661,17 +2661,17 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện kiểm kê tài sản thiết bị định kỳ; đề xuất mua sắm bổ sung thiết bị dạy học tối thiểu và thanh lý đồ hỏng</t>
+          <t>Kiểm tra thể thức, lấy số, phát hành các quyết định phân công chuyên môn, kế hoạch khai giảng và văn bản đầu năm học</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E69" s="9" t="n">
@@ -2685,27 +2685,27 @@
       </c>
       <c r="H69" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm kê thiết bị dạy học cuối kỳ/năm</t>
+          <t>Sổ theo dõi văn bản đi tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Quản lý kho sách, cấp phát SGK, SGV và tài liệu tham khảo cho giáo viên, học sinh ngay đầu năm học mới</t>
+          <t>Quản lý con dấu, chứng thư số; thực hiện đóng dấu giấy xác nhận học sinh, chứng chỉ cho học sinh đầu năm đúng quy định</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="E70" s="9" t="n">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>Sổ đăng ký cá biệt, sổ mượn trả sách thư viện</t>
+          <t>Sổ cấp giấy xác nhận học sinh năm học 2026-2027</t>
         </is>
       </c>
     </row>
@@ -2729,17 +2729,17 @@
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức hoạt động hưởng ứng Ngày Sách và Văn hóa đọc Việt Nam, tuyên truyền giới thiệu sách hay cho học sinh</t>
+          <t>Mở sổ quỹ tiền mặt năm học 2026 - 2027, ghi chép thu chi quỹ tháng 9 chính xác, thực hiện kiểm kê quỹ cuối tháng</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>30/04/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E71" s="9" t="n">
@@ -2753,27 +2753,27 @@
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch và báo cáo tổ chức Ngày hội đọc sách năm học</t>
+          <t>Sổ quỹ tiền mặt tháng 9/2026 có xác nhận của Kế toán và Hiệu trưởng</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Quản lý tủ thuốc y tế trường học; lập kế hoạch và tổ chức sơ cứu, chăm sóc sức khỏe ban đầu cho học sinh và cán bộ</t>
+          <t>Lập kế hoạch sử dụng phòng học bộ môn và chuẩn bị đầy đủ thiết bị, hóa chất phục vụ các tiết dạy thực hành tháng 9</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E72" s="9" t="n">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi khám chữa bệnh và cấp phát thuốc sơ cứu</t>
+          <t>Sổ mượn trả thiết bị dạy học tháng 9/2026</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Tuyên truyền phòng chống dịch bệnh theo mùa, vệ sinh an toàn thực phẩm, vận động học sinh tham gia BHYT đạt 100%</t>
+          <t>Kiểm tra tủ thuốc y tế, bổ sung bông băng thuốc thiết yếu và lập kế hoạch chăm sóc sức khỏe học sinh đầu năm học mới</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="E73" s="9" t="n">
@@ -2821,27 +2821,27 @@
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo y tế học đường và tỷ lệ học sinh tham gia BHYT đạt 100%</t>
+          <t>Kế hoạch y tế học đường năm học 2026-2027 và danh mục thuốc</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Quản trị, vận hành hệ thống mạng internet, phòng máy tính tin học, bảo đảm kết nối thông suốt phục vụ học tập và thi</t>
+          <t>Tuyên truyền phòng chống sốt xuất huyết, dịch bệnh mùa thu và phối hợp vận động học sinh tham gia BHYT đạt 100%</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E74" s="9" t="n">
@@ -2855,17 +2855,17 @@
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>Nhật ký vận hành phòng máy tính và bảo dưỡng định kỳ hệ thống mạng</t>
+          <t>Báo cáo công tác BHYT học sinh tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Quản trị kỹ thuật cổng thông tin điện tử (website) nhà trường, hỗ trợ kỹ thuật phần mềm CSDL, học bạ số và chữ ký số</t>
+          <t>Đưa tin bài, hình ảnh Lễ Khai giảng năm học 2026 - 2027 lên website trường; sao lưu an toàn CSDL tháng 9/2026</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>31/05/2027</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E75" s="9" t="n">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo an toàn thông tin và dữ liệu sao lưu định kỳ hệ thống</t>
+          <t>Link bài viết trên website trường và file nhật ký sao lưu hệ thống</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bo sung Thang 5/2026: CBQL 33cv GV 27cv NV 30cv - Tong 90 cong viec giai doan T5-T9/2026 - Them bo loc theo thang
</commit_message>
<xml_diff>
--- a/public/downloads/Import công việc.xlsx
+++ b/public/downloads/Import công việc.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mẫu import" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="SPCV" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mẫu import" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPCV" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L75"/>
+  <dimension ref="A2:L199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -621,17 +621,17 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Tổng hợp kết quả đánh giá, xếp loại chất lượng viên chức, người lao động cuối năm học 2025 - 2026 theo Nghị định 90/2020 &amp; 48/2023</t>
+          <t>Chỉ đạo hoàn thành chương trình dạy học học kỳ II, tổ chức ôn tập và kiểm tra đánh giá cuối học kỳ II năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
@@ -645,27 +645,27 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp Hội đồng đánh giá xếp loại viên chức năm học 2025-2026</t>
+          <t>Kế hoạch kiểm tra cuối học kỳ II năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Quyết định công nhận kết quả đánh giá, xếp loại viên chức, người lao động và công khai toàn trường</t>
+          <t>Chỉ đạo thu nhận, kiểm tra, rà soát hồ sơ và hoàn thành dữ liệu đăng ký dự thi tốt nghiệp THPT năm 2026 trên Cổng Quản lý thi</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
+          <t>N2_1102 - Tổ chức đăng ký dự thi và nhận dữ liệu đăng ký dự thi tốt nghiệp THPT; đăng ký dự thi đăng ký xét tuyển sinh đại học, cao đẳng g</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
@@ -679,7 +679,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Quyết định số 85/QĐ-THPT công nhận kết quả xếp loại</t>
+          <t>Danh sách thí sinh đăng ký dự thi tốt nghiệp THPT 2026 đã duyệt</t>
         </is>
       </c>
     </row>
@@ -689,17 +689,17 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo thẩm định hồ sơ thi đua, sáng kiến kinh nghiệm của CBGVNV đề nghị công nhận LĐTT, CSTĐ cơ sở năm học 2025 - 2026</t>
+          <t>Chỉ đạo rà soát, kiểm tra học bạ số và đồng bộ dữ liệu điểm học tập cấp THPT lên Hệ thống Quản lý thi của Bộ GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
+          <t>N2_1095 - Chỉ đạo, tổ chức rà soát kết quả điểm học tập cấp THPT (học bạ) trên Hệ thống Quản lý thi theo Chỉ đạo của Bộ GDĐT</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
@@ -713,27 +713,27 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Biên bản thẩm định hồ sơ sáng kiến kinh nghiệm và thi đua</t>
+          <t>Biên bản rà soát học bạ điện tử khối 12 trên hệ thống thi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức họp Hội đồng Thi đua - Khen thưởng nhà trường xét duyệt danh hiệu và hoàn thiện tờ trình nộp Sở GD&amp;ĐT</t>
+          <t>Tổ chức kỳ thi thử tốt nghiệp THPT năm 2026 đợt cuối cho học sinh lớp 12, phân tích phổ điểm để điều chỉnh phương pháp ôn tập</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
+          <t>N2_1091 - Tổ chức thi thử tốt nghiệp THPT năm 2026 (ra đề, in sao đề thi)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
@@ -747,7 +747,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Tờ trình số 28/TTr-THPT đề nghị khen thưởng năm học 2025-2026</t>
+          <t>Báo cáo phân tích phổ điểm thi thử tốt nghiệp THPT 2026</t>
         </is>
       </c>
     </row>
@@ -757,17 +757,17 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Rà soát, chuẩn bị đầy đủ phòng thi, camera giám sát, thiết bị PCCC, phòng bảo quản đề thi, bài thi phục vụ Điểm thi tốt nghiệp THPT năm 2026</t>
+          <t>Chỉ đạo tổng kết đánh giá xếp loại học sinh, tổng kết công tác chuyên môn và lập báo cáo thống kê cuối năm học 2025 - 2026 nộp Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
+          <t>N2_1126 - Tổng hợp báo cáo thống kê kỳ cuối năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>20/06/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
@@ -781,27 +781,27 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm tra điều kiện CSVC Điểm thi tốt nghiệp THPT năm 2026</t>
+          <t>Báo cáo tổng kết năm học 2025-2026 trường THPT Phục Hòa</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Phối hợp với chính quyền địa phương, công an, y tế bảo đảm an ninh trật tự, an toàn giao thông và phòng chống dịch bệnh kỳ thi tốt nghiệp</t>
+          <t>Xây dựng Kế hoạch và chỉ đạo tổ chức Lễ Bế giảng năm học 2025 - 2026, Lễ Tri ân và Trưởng thành cho học sinh niên khóa 2023 - 2026</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
+          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
@@ -815,7 +815,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch phối hợp liên ngành bảo đảm an ninh trật tự kỳ thi</t>
+          <t>Kế hoạch tổ chức Lễ Bế giảng và Tri ân trưởng thành năm học 2025-2026</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Thành lập Hội đồng tuyển sinh lớp 10 THPT năm học 2026 - 2027; ban hành Thông báo hướng dẫn tuyển sinh</t>
+          <t>Tổ chức họp giao ban BGH và họp Hội đồng sư phạm tháng 5/2026 rà soát nhiệm vụ kết thúc năm học và triển khai hoạt động hè</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
@@ -849,27 +849,27 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Quyết định thành lập HĐTS và Thông báo số 12/TB-THPT tuyển sinh lớp 10</t>
+          <t>Biên bản họp Hội đồng sư phạm tháng 5/2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo thu nhận hồ sơ, xét tuyển, hoàn thành duyệt danh sách trúng tuyển lớp 10 trình Sở GD&amp;ĐT phê duyệt</t>
+          <t>Duy trì lịch tiếp công dân định kỳ tháng 5/2026, lắng nghe và giải quyết kịp thời thắc mắc của phụ huynh học sinh cuối năm học</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
+          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>25/07/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="E16" s="9" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Danh sách học sinh trúng tuyển lớp 10 đã được Sở GD&amp;ĐT phê duyệt</t>
+          <t>Sổ theo dõi tiếp công dân tháng 5/2026</t>
         </is>
       </c>
     </row>
@@ -893,17 +893,17 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch bồi dưỡng chính trị hè năm 2026 và bồi dưỡng chuyên môn nghiệp vụ cho cán bộ quản lý, giáo viên</t>
+          <t>Tổng hợp kết quả đánh giá, xếp loại chất lượng viên chức, người lao động cuối năm học 2025 - 2026 theo Nghị định 90/2020 &amp; 48/2023</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
@@ -917,27 +917,27 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch số 45/KH-THPT bồi dưỡng chính trị và chuyên môn hè 2026</t>
+          <t>Biên bản họp Hội đồng đánh giá xếp loại viên chức năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo rà soát, xét duyệt quyết toán thu chi ngân sách 6 tháng đầu năm 2026 và đối chiếu kho bạc</t>
+          <t>Ban hành Quyết định công nhận kết quả đánh giá, xếp loại viên chức, người lao động và công khai toàn trường</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>N2_1158 - Xét duyệt quyết toán ngân sách Nhà nước hàng năm</t>
+          <t>N2_1046 - Tham mưu công tác đánh giá, xếp loại</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="E18" s="9" t="n">
@@ -951,27 +951,27 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo quyết toán tài chính ngân sách 6 tháng đầu năm 2026</t>
+          <t>Quyết định số 85/QĐ-THPT công nhận kết quả xếp loại</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Cử cán bộ quản lý, giáo viên tham gia đầy đủ các lớp tập huấn SGK, phương pháp giảng dạy và ứng dụng AI do Sở GD&amp;ĐT tổ chức</t>
+          <t>Chỉ đạo thẩm định hồ sơ thi đua, sáng kiến kinh nghiệm của CBGVNV đề nghị công nhận LĐTT, CSTĐ cơ sở năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
@@ -985,27 +985,27 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>Quyết định cử cán bộ, giáo viên dự tập huấn hè năm 2026</t>
+          <t>Biên bản thẩm định hồ sơ sáng kiến kinh nghiệm và thi đua</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra, nghiệm thu công tác sửa chữa phòng học, bàn ghế, hệ thống điện nước, mái che và vệ sinh khuôn viên trường trong hè</t>
+          <t>Tổ chức họp Hội đồng Thi đua - Khen thưởng nhà trường xét duyệt danh hiệu và hoàn thiện tờ trình nộp Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
+          <t>N1_576 - Tiếp nhận, thẩm định hồ sơ đề nghị xét tặng thưởng danh hiệu Lao động tiên tiến, Chiến sỹ thi đua cơ sở và hồ sơ trình khen thưở</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="E20" s="9" t="n">
@@ -1019,27 +1019,27 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Biên bản nghiệm thu tu sửa cơ sở vật chất hè 2026</t>
+          <t>Tờ trình số 28/TTr-THPT đề nghị khen thưởng năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Rà soát, mua sắm bổ sung thiết bị dạy học tối thiểu, sách thư viện và hóa chất thí nghiệm chuẩn bị năm học mới 2026 - 2027</t>
+          <t>Rà soát, chuẩn bị đầy đủ phòng thi, camera giám sát, thiết bị PCCC, phòng bảo quản đề thi, bài thi phục vụ Điểm thi tốt nghiệp THPT năm 2026</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
+          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
@@ -1053,27 +1053,27 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>Hợp đồng mua sắm thiết bị dạy học và sách thư viện</t>
+          <t>Biên bản kiểm tra điều kiện CSVC Điểm thi tốt nghiệp THPT năm 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Quyết định phân công nhiệm vụ cán bộ quản lý, phân công chuyên môn giáo viên và biên chế học sinh các lớp năm học 2026 - 2027</t>
+          <t>Phối hợp với chính quyền địa phương, công an, y tế bảo đảm an ninh trật tự, an toàn giao thông và phòng chống dịch bệnh kỳ thi tốt nghiệp</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
+          <t>N1_580 - Phối hợp chuẩn bị các điều kiện về cơ sở vật chất, trang thiết bị phục vụ cho công tác tổ chức kỳ thi tuyển sinh 10; thi tốt ngh</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>20/08/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="E22" s="9" t="n">
@@ -1087,27 +1087,27 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>Quyết định số 102/QĐ-THPT về phân công nhiệm vụ năm học 2026-2027</t>
+          <t>Kế hoạch phối hợp liên ngành bảo đảm an ninh trật tự kỳ thi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo tổ chức ngày tựu trường, đón học sinh lớp 10 và tổ chức tuần sinh hoạt tập thể đầu năm học 2026 - 2027</t>
+          <t>Thành lập Hội đồng tuyển sinh lớp 10 THPT năm học 2026 - 2027; ban hành Thông báo hướng dẫn tuyển sinh</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
+          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
@@ -1121,27 +1121,27 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch tựu trường và tuần sinh hoạt tập thể học sinh đầu năm</t>
+          <t>Quyết định thành lập HĐTS và Thông báo số 12/TB-THPT tuyển sinh lớp 10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch và chỉ đạo tổ chức Lễ Khai giảng năm học mới 2026 - 2027 trang trọng, ý nghĩa, an toàn và tiết kiệm</t>
+          <t>Chỉ đạo thu nhận hồ sơ, xét tuyển, hoàn thành duyệt danh sách trúng tuyển lớp 10 trình Sở GD&amp;ĐT phê duyệt</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>N3_666 - Kế hoạch tham dự Lễ Khai giảng năm học 2026 - 2027 tại các cơ sở giáo dục trên địa bàn tỉnh Cao Bằng</t>
+          <t>N2_1097 - Hướng dẫn tuyển sinh lớp 10 trung học phổ thông năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="E24" s="9" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch tổ chức Lễ Khai giảng năm học 2026-2027</t>
+          <t>Danh sách học sinh trúng tuyển lớp 10 đã được Sở GD&amp;ĐT phê duyệt</t>
         </is>
       </c>
     </row>
@@ -1165,17 +1165,17 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng và ban hành Kế hoạch giáo dục nhà trường, kế hoạch thực hiện nhiệm vụ trọng tâm năm học 2026 - 2027</t>
+          <t>Xây dựng Kế hoạch bồi dưỡng chính trị hè năm 2026 và bồi dưỡng chuyên môn nghiệp vụ cho cán bộ quản lý, giáo viên</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
@@ -1189,27 +1189,27 @@
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch giáo dục nhà trường năm học 2026-2027</t>
+          <t>Kế hoạch số 45/KH-THPT bồi dưỡng chính trị và chuyên môn hè 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Phê duyệt kế hoạch giáo dục của các tổ chuyên môn, tổ văn phòng và các bộ phận trong nhà trường năm học 2026 - 2027</t>
+          <t>Chỉ đạo rà soát, xét duyệt quyết toán thu chi ngân sách 6 tháng đầu năm 2026 và đối chiếu kho bạc</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N2_1158 - Xét duyệt quyết toán ngân sách Nhà nước hàng năm</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="E26" s="9" t="n">
@@ -1223,27 +1223,27 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch năm học các tổ TN, XH, VP đã phê duyệt</t>
+          <t>Báo cáo quyết toán tài chính ngân sách 6 tháng đầu năm 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo tổ chức thành công Hội nghị cán bộ, viên chức, người lao động năm học 2026 - 2027</t>
+          <t>Cử cán bộ quản lý, giáo viên tham gia đầy đủ các lớp tập huấn SGK, phương pháp giảng dạy và ứng dụng AI do Sở GD&amp;ĐT tổ chức</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Nghị quyết Hội nghị CBVC-NLĐ năm học 2026-2027</t>
+          <t>Quyết định cử cán bộ, giáo viên dự tập huấn hè năm 2026</t>
         </is>
       </c>
     </row>
@@ -1267,17 +1267,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng lịch công tác tuần, tháng 9 và chương trình điều hành tổng thể hoạt động sư phạm toàn trường</t>
+          <t>Kiểm tra, nghiệm thu công tác sửa chữa phòng học, bàn ghế, hệ thống điện nước, mái che và vệ sinh khuôn viên trường trong hè</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
+          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E28" s="9" t="n">
@@ -1291,27 +1291,27 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Lịch công tác tuần tháng 9/2026 đăng tải trên cổng thông tin điện tử</t>
+          <t>Biên bản nghiệm thu tu sửa cơ sở vật chất hè 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức họp giao ban BGH và họp Hội đồng sư phạm tháng 9/2026 đánh giá triển khai nhiệm vụ năm học mới</t>
+          <t>Rà soát, mua sắm bổ sung thiết bị dạy học tối thiểu, sách thư viện và hóa chất thí nghiệm chuẩn bị năm học mới 2026 - 2027</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+          <t>N3_684 - Tham mưu triển khai công tác thuộc lĩnh vực Cơ sở vật chất</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
@@ -1325,27 +1325,27 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp Hội đồng sư phạm tháng 9/2026</t>
+          <t>Hợp đồng mua sắm thiết bị dạy học và sách thư viện</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra, đôn đốc tiến độ thực hiện chương trình giảng dạy và nền nếp chuyên môn tháng 9</t>
+          <t>Ban hành Quyết định phân công nhiệm vụ cán bộ quản lý, phân công chuyên môn giáo viên và biên chế học sinh các lớp năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
@@ -1359,27 +1359,27 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo kiểm tra nền nếp dạy học tháng 9/2026</t>
+          <t>Quyết định số 102/QĐ-THPT về phân công nhiệm vụ năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Tổng hợp số liệu đầu năm, kiểm tra việc ổn định nền nếp dạy học tháng 9 và báo cáo Sở GD&amp;ĐT đúng thời hạn</t>
+          <t>Chỉ đạo tổ chức ngày tựu trường, đón học sinh lớp 10 và tổ chức tuần sinh hoạt tập thể đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
+          <t>N1_585 - Chỉ đạo việc thực hiện các nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="E31" s="9" t="n">
@@ -1393,27 +1393,27 @@
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo tình hình triển khai nhiệm vụ đầu năm học gửi Sở GD&amp;ĐT</t>
+          <t>Kế hoạch tựu trường và tuần sinh hoạt tập thể học sinh đầu năm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Chỉ đạo triển khai công tác tuyên truyền phổ biến pháp luật, an toàn giao thông và cam kết an ninh trật tự trường học tháng 9</t>
+          <t>Xây dựng Kế hoạch và chỉ đạo tổ chức Lễ Khai giảng năm học mới 2026 - 2027 trang trọng, ý nghĩa, an toàn và tiết kiệm</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
+          <t>N3_666 - Kế hoạch tham dự Lễ Khai giảng năm học 2026 - 2027 tại các cơ sở giáo dục trên địa bàn tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>Bản cam kết an toàn giao thông và phòng chống bạo lực học đường</t>
+          <t>Kế hoạch tổ chức Lễ Khai giảng năm học 2026-2027</t>
         </is>
       </c>
     </row>
@@ -1437,17 +1437,17 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Ban hành Thông báo Lịch tiếp công dân năm học 2026 - 2027; tiếp nhận và giải quyết kịp thời phản ánh của phụ huynh đầu năm học</t>
+          <t>Xây dựng và ban hành Kế hoạch giáo dục nhà trường, kế hoạch thực hiện nhiệm vụ trọng tâm năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
@@ -1461,27 +1461,27 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>Thông báo lịch tiếp công dân năm học 2026-2027 và sổ tiếp dân</t>
+          <t>Kế hoạch giáo dục nhà trường năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Hoàn thành chấm bài, vào điểm, tổng kết đánh giá xếp loại học sinh cuối năm học 2025 - 2026 trên phần mềm VnEdu</t>
+          <t>Phê duyệt kế hoạch giáo dục của các tổ chuyên môn, tổ văn phòng và các bộ phận trong nhà trường năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
@@ -1495,27 +1495,27 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>Sổ điểm điện tử năm học 2025-2026 trên hệ thống VnEdu</t>
+          <t>Kế hoạch năm học các tổ TN, XH, VP đã phê duyệt</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện nhiệm vụ coi thi, chấm thi kỳ thi tuyển sinh lớp 10 THPT và kỳ thi tốt nghiệp THPT năm 2026 theo điều động của Sở</t>
+          <t>Chỉ đạo tổ chức thành công Hội nghị cán bộ, viên chức, người lao động năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+          <t>N3_668 - Quyết định ban hành Kế hoạch nhiệm vụ, giải pháp trọng tâm năm học 2026 - 2027 của ngành Giáo dục tỉnh Cao Bằng</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>Quyết định điều động cán bộ coi thi, chấm thi của Sở GD&amp;ĐT</t>
+          <t>Nghị quyết Hội nghị CBVC-NLĐ năm học 2026-2027</t>
         </is>
       </c>
     </row>
@@ -1539,17 +1539,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Hoàn thiện hồ sơ sáng kiến kinh nghiệm, hồ sơ minh chứng đề nghị đánh giá xếp loại viên chức cuối năm học 2025 - 2026</t>
+          <t>Xây dựng lịch công tác tuần, tháng 9 và chương trình điều hành tổng thể hoạt động sư phạm toàn trường</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+          <t>N1_610 - Chủ trì xây dựng kế hoạch, chương trình công tác của Phòng</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo sáng kiến kinh nghiệm và phiếu tự đánh giá viên chức</t>
+          <t>Lịch công tác tuần tháng 9/2026 đăng tải trên cổng thông tin điện tử</t>
         </is>
       </c>
     </row>
@@ -1573,17 +1573,17 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Tham gia đầy đủ lớp bồi dưỡng chính trị hè năm 2026 và hoàn thành bài thu hoạch đạt yêu cầu</t>
+          <t>Tổ chức họp giao ban BGH và họp Hội đồng sư phạm tháng 9/2026 đánh giá triển khai nhiệm vụ năm học mới</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>25/07/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>Bài thu hoạch bồi dưỡng chính trị hè 2026</t>
+          <t>Biên bản họp Hội đồng sư phạm tháng 9/2026</t>
         </is>
       </c>
     </row>
@@ -1607,17 +1607,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Hoàn thành khóa tập huấn chuyên môn, bồi dưỡng SGK và đổi mới phương pháp dạy học theo CT GDPT 2018 trong hè</t>
+          <t>Kiểm tra, đôn đốc tiến độ thực hiện chương trình giảng dạy và nền nếp chuyên môn tháng 9</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E38" s="9" t="n">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>Giấy chứng nhận / kết quả hoàn thành tập huấn bồi dưỡng hè 2026</t>
+          <t>Báo cáo kiểm tra nền nếp dạy học tháng 9/2026</t>
         </is>
       </c>
     </row>
@@ -1641,17 +1641,17 @@
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch dạy học môn học cá nhân năm học 2026 - 2027 nộp Tổ trưởng chuyên môn phê duyệt</t>
+          <t>Tổng hợp số liệu đầu năm, kiểm tra việc ổn định nền nếp dạy học tháng 9 và báo cáo Sở GD&amp;ĐT đúng thời hạn</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="E39" s="9" t="n">
@@ -1665,27 +1665,27 @@
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch dạy học cá nhân năm học 2026-2027 có xác nhận của Tổ trưởng</t>
+          <t>Báo cáo tình hình triển khai nhiệm vụ đầu năm học gửi Sở GD&amp;ĐT</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Nhận lớp chủ nhiệm, tổ chức cho học sinh tựu trường, ổn định tổ chức lớp và phổ biến nội quy học sinh</t>
+          <t>Chỉ đạo triển khai công tác tuyên truyền phổ biến pháp luật, an toàn giao thông và cam kết an ninh trật tự trường học tháng 9</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N2_1131 - Tổng hợp báo cáo tình hình triển khai nhiệm vụ đầu năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E40" s="9" t="n">
@@ -1699,27 +1699,27 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp lớp đầu năm và danh sách ban cán sự lớp</t>
+          <t>Bản cam kết an toàn giao thông và phòng chống bạo lực học đường</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Chuẩn bị trang phục, hướng dẫn học sinh tham gia Lễ Khai giảng năm học 2026 - 2027 trang nghiêm, đầy đủ quân số</t>
+          <t>Ban hành Thông báo Lịch tiếp công dân năm học 2026 - 2027; tiếp nhận và giải quyết kịp thời phản ánh của phụ huynh đầu năm học</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N1_572 - Tiếp công dân định kỳ cùng Giám đốc Sở GDĐT</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
@@ -1733,27 +1733,27 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>Sổ chủ nhiệm ghi nhận quân số dự Khai giảng 100%</t>
+          <t>Thông báo lịch tiếp công dân năm học 2026-2027 và sổ tiếp dân</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Tổ chức Hội nghị Ban đại diện Cha mẹ học sinh lớp đầu năm học 2026 - 2027; lập biên bản họp đúng quy định</t>
+          <t>Hoàn thành nội dung chương trình giảng dạy học kỳ II theo phân phối chương trình, bảo đảm đúng tiến độ quy định</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
@@ -1767,27 +1767,27 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp phụ huynh học sinh đầu năm học 2026-2027</t>
+          <t>Sổ ghi đầu bài các lớp hoàn thành chương trình tuần 35</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Cập nhật hồ sơ học sinh, hoàn thiện cơ sở dữ liệu lý lịch và thông tin liên lạc của học sinh trên hệ thống VnEdu</t>
+          <t>Thực hiện ra đề, coi thi, chấm bài kiểm tra cuối học kỳ II theo đúng ma trận đặc tả; nhập điểm đầy đủ lên VnEdu</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
@@ -1801,27 +1801,27 @@
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>Dữ liệu hồ sơ học sinh lớp chủ nhiệm trên hệ thống CSDL trường</t>
+          <t>Bảng điểm kiểm tra cuối học kỳ II trên hệ thống VnEdu</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Soạn Kế hoạch bài dạy (giáo án) các tuần học tháng 9/2026 đúng chuẩn Công văn 5512/BGDĐT, tích hợp năng lực số và AI</t>
+          <t>Thực hiện coi thi, chấm thi thử tốt nghiệp THPT 2026 môn phụ trách, hướng dẫn học sinh sửa bài và ôn tập củng cố kiến thức</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N2_1091 - Tổ chức thi thử tốt nghiệp THPT năm 2026 (ra đề, in sao đề thi)</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="E44" s="9" t="n">
@@ -1835,27 +1835,27 @@
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>Giáo án các tuần 1, 2, 3, 4 tháng 9 lưu trên hệ thống CSDL giáo án</t>
+          <t>Bảng phân tích kết quả bài thi thử của học sinh</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế bài giảng điện tử và học liệu số tương tác phục vụ dạy học các chuyên đề đầu năm học mới</t>
+          <t>Hoàn thành đánh giá xếp loại học lực, hạnh kiểm/kết quả học tập và rèn luyện của học sinh lớp chủ nhiệm cuối năm trên VnEdu</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>N1_550 - Soạn thảo văn bản hành chính</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
@@ -1869,27 +1869,27 @@
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>Link bài giảng điện tử và học liệu số tải lên thư viện trường</t>
+          <t>Sổ tổng hợp kết quả đánh giá học sinh năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện nghiêm túc thời khóa biểu tháng 9/2026, lên lớp đúng giờ, duy trì tốt nền nếp và kỷ luật dạy học</t>
+          <t>Tổ chức họp Ban đại diện Cha mẹ học sinh lớp cuối năm học 2025 - 2026, thông báo kết quả học tập và phối hợp quản lý học sinh hè</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="E46" s="9" t="n">
@@ -1903,27 +1903,27 @@
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>Sổ đầu bài các lớp giảng dạy tháng 9/2026</t>
+          <t>Biên bản họp phụ huynh học sinh cuối năm học 2025-2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Tham gia các buổi sinh hoạt tổ chuyên môn đầu năm học: thống nhất ma trận đề, kế hoạch giáo dục và quy chế tổ</t>
+          <t>Hoàn thiện báo cáo kết quả thực hiện Sáng kiến kinh nghiệm / Đề tài NCKH sư phạm ứng dụng năm học 2025 - 2026 nộp Hội đồng cơ sở</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
@@ -1937,27 +1937,27 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Biên bản họp tổ chuyên môn tháng 9/2026</t>
+          <t>Bản báo cáo kết quả đề tài sáng kiến kinh nghiệm cá nhân</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện dự giờ đồng nghiệp tháng 9 theo kế hoạch tổ chuyên môn (đạt 2 tiết/tháng), trao đổi kinh nghiệm sư phạm</t>
+          <t>Tự đánh giá Chuẩn nghề nghiệp giáo viên cơ sở giáo dục phổ thông năm học 2025 - 2026 theo Thông tư 20/2018/TT-BGDĐT và cập nhật TEMIS</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="E48" s="9" t="n">
@@ -1971,17 +1971,17 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>Sổ dự giờ giáo viên có nhận xét và đánh giá tiết dạy</t>
+          <t>Phiếu tự đánh giá Chuẩn nghề nghiệp giáo viên trên hệ thống TEMIS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện kiểm tra đánh giá thường xuyên học sinh theo đúng kế hoạch; chấm bài và vào điểm VnEdu kịp thời</t>
+          <t>Hoàn thành chấm bài, vào điểm, tổng kết đánh giá xếp loại học sinh cuối năm học 2025 - 2026 trên phần mềm VnEdu</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
@@ -2005,27 +2005,27 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>Điểm kiểm tra thường xuyên tháng 9 cập nhật trên VnEdu</t>
+          <t>Sổ điểm điện tử năm học 2025-2026 trên hệ thống VnEdu</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Khảo sát chất lượng đầu năm, phát hiện và lập danh sách học sinh năng khiếu để bồi dưỡng đội tuyển HSG môn phụ trách</t>
+          <t>Thực hiện nhiệm vụ coi thi, chấm thi kỳ thi tuyển sinh lớp 10 THPT và kỳ thi tốt nghiệp THPT năm 2026 theo điều động của Sở</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="E50" s="9" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>Danh sách đội tuyển HSG và Kế hoạch bồi dưỡng HSG</t>
+          <t>Quyết định điều động cán bộ coi thi, chấm thi của Sở GD&amp;ĐT</t>
         </is>
       </c>
     </row>
@@ -2049,17 +2049,17 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Lập danh sách học sinh học lực yếu kém đầu năm học để xây dựng phương án dạy phụ đạo, kèm cặp nâng cao chất lượng</t>
+          <t>Hoàn thiện hồ sơ sáng kiến kinh nghiệm, hồ sơ minh chứng đề nghị đánh giá xếp loại viên chức cuối năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="E51" s="9" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch phụ đạo học sinh có kết quả khảo sát đầu năm thấp</t>
+          <t>Báo cáo sáng kiến kinh nghiệm và phiếu tự đánh giá viên chức</t>
         </is>
       </c>
     </row>
@@ -2083,17 +2083,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Đăng ký tên đề tài Sáng kiến kinh nghiệm hoặc Đề tài nghiên cứu khoa học sư phạm ứng dụng năm học 2026 - 2027</t>
+          <t>Tham gia đầy đủ lớp bồi dưỡng chính trị hè năm 2026 và hoàn thành bài thu hoạch đạt yêu cầu</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="E52" s="9" t="n">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Phiếu đăng ký đề tài SKKN năm học 2026-2027 nộp Tổ chuyên môn</t>
+          <t>Bài thu hoạch bồi dưỡng chính trị hè 2026</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Xây dựng Kế hoạch tự bồi dưỡng thường xuyên cá nhân năm học 2026 - 2027 theo quy định của Bộ và Sở GD&amp;ĐT</t>
+          <t>Hoàn thành khóa tập huấn chuyên môn, bồi dưỡng SGK và đổi mới phương pháp dạy học theo CT GDPT 2018 trong hè</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="E53" s="9" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>Bản kế hoạch tự học, bồi dưỡng thường xuyên năm học 2026-2027</t>
+          <t>Giấy chứng nhận / kết quả hoàn thành tập huấn bồi dưỡng hè 2026</t>
         </is>
       </c>
     </row>
@@ -2151,17 +2151,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Rút dự toán thanh toán tiền lương, các khoản phụ cấp tháng 6/2026 cho cán bộ, giáo viên, nhân viên đúng thời hạn</t>
+          <t>Xây dựng Kế hoạch dạy học môn học cá nhân năm học 2026 - 2027 nộp Tổ trưởng chuyên môn phê duyệt</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E54" s="9" t="n">
@@ -2175,27 +2175,27 @@
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>Giấy rút dự toán ngân sách và bảng thanh toán lương tháng 6/2026</t>
+          <t>Kế hoạch dạy học cá nhân năm học 2026-2027 có xác nhận của Tổ trưởng</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Tiếp nhận, đăng ký, chuyển giao kịp thời văn bản chỉ đạo của Sở về thi tốt nghiệp THPT và tuyển sinh lớp 10 năm 2026</t>
+          <t>Nhận lớp chủ nhiệm, tổ chức cho học sinh tựu trường, ổn định tổ chức lớp và phổ biến nội quy học sinh</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>20/06/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="E55" s="9" t="n">
@@ -2209,27 +2209,27 @@
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi văn bản đến tháng 6/2026 trên iOffice</t>
+          <t>Biên bản họp lớp đầu năm và danh sách ban cán sự lớp</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Chuẩn bị cơ số thuốc, vật tư y tế, phòng y tế phục vụ Điểm thi tốt nghiệp THPT năm 2026 tại trường an toàn</t>
+          <t>Chuẩn bị trang phục, hướng dẫn học sinh tham gia Lễ Khai giảng năm học 2026 - 2027 trang nghiêm, đầy đủ quân số</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E56" s="9" t="n">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm tra điều kiện y tế phục vụ kỳ thi tốt nghiệp 2026</t>
+          <t>Sổ chủ nhiệm ghi nhận quân số dự Khai giảng 100%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Bảo dưỡng, kiểm tra hệ thống máy vi tính, đường truyền internet, camera giám sát phục vụ thi tốt nghiệp THPT 2026</t>
+          <t>Tổ chức Hội nghị Ban đại diện Cha mẹ học sinh lớp đầu năm học 2026 - 2027; lập biên bản họp đúng quy định</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>20/06/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E57" s="9" t="n">
@@ -2277,27 +2277,27 @@
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>Nhật ký kiểm tra thiết bị CNTT phục vụ kỳ thi</t>
+          <t>Biên bản họp phụ huynh học sinh đầu năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Thu hồi SGK, tài liệu tham khảo cho mượn năm học 2025 - 2026; xử lý kỹ thuật và sắp xếp lại kho sách thư viện</t>
+          <t>Cập nhật hồ sơ học sinh, hoàn thiện cơ sở dữ liệu lý lịch và thông tin liên lạc của học sinh trên hệ thống VnEdu</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>28/06/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E58" s="9" t="n">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi mượn trả sách thư viện cuối năm</t>
+          <t>Dữ liệu hồ sơ học sinh lớp chủ nhiệm trên hệ thống CSDL trường</t>
         </is>
       </c>
     </row>
@@ -2321,17 +2321,17 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Thực hiện đối chiếu số dư tài khoản tiền gửi và hạn mức kinh phí 6 tháng đầu năm 2026 với Kho bạc Nhà nước</t>
+          <t>Soạn Kế hoạch bài dạy (giáo án) các tuần học tháng 9/2026 đúng chuẩn Công văn 5512/BGDĐT, tích hợp năng lực số và AI</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E59" s="9" t="n">
@@ -2345,27 +2345,27 @@
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>Biên bản đối chiếu tài khoản với KBNN kỳ 6 tháng đầu năm 2026</t>
+          <t>Giáo án các tuần 1, 2, 3, 4 tháng 9 lưu trên hệ thống CSDL giáo án</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Lập báo cáo tài chính và báo cáo quyết toán ngân sách nhà nước 6 tháng đầu năm 2026 nộp Sở GD&amp;ĐT</t>
+          <t>Thiết kế bài giảng điện tử và học liệu số tương tác phục vụ dạy học các chuyên đề đầu năm học mới</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+          <t>N1_550 - Soạn thảo văn bản hành chính</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="E60" s="9" t="n">
@@ -2379,27 +2379,27 @@
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo quyết toán ngân sách 6 tháng đầu năm 2026</t>
+          <t>Link bài giảng điện tử và học liệu số tải lên thư viện trường</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Tiếp nhận hồ sơ, sao lục học bạ và cấp phát giấy chứng nhận tốt nghiệp tạm thời cho học sinh khối 12 năm 2026</t>
+          <t>Thực hiện nghiêm túc thời khóa biểu tháng 9/2026, lên lớp đúng giờ, duy trì tốt nền nếp và kỷ luật dạy học</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E61" s="9" t="n">
@@ -2413,27 +2413,27 @@
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>Sổ cấp phát văn bằng chứng chỉ, giấy chứng nhận tốt nghiệp tạm thời</t>
+          <t>Sổ đầu bài các lớp giảng dạy tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Thu thập, phân loại và lưu trữ toàn bộ hồ sơ thi tốt nghiệp THPT 2026, hồ sơ tuyển sinh 10 và hồ sơ thi đua năm học 2025 - 2026</t>
+          <t>Tham gia các buổi sinh hoạt tổ chuyên môn đầu năm học: thống nhất ma trận đề, kế hoạch giáo dục và quy chế tổ</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>N1_604 - Thu thập hồ sơ tài liệu vào kho lưu trữ, phục vụ khai thác, sử dụng tài liệu lưu trữ</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E62" s="9" t="n">
@@ -2447,27 +2447,27 @@
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>Mục lục hồ sơ tài liệu nộp lưu trữ cơ quan đợt hè 2026</t>
+          <t>Biên bản họp tổ chuyên môn tháng 9/2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Chi trả kịp thời tiền làm nhiệm vụ coi thi, chấm thi và tiền phụ cấp làm việc hè cho cán bộ, giáo viên đúng danh sách</t>
+          <t>Thực hiện dự giờ đồng nghiệp tháng 9 theo kế hoạch tổ chuyên môn (đạt 2 tiết/tháng), trao đổi kinh nghiệm sư phạm</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="E63" s="9" t="n">
@@ -2481,27 +2481,27 @@
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>Bảng thanh toán tiền làm nhiệm vụ thi có chữ ký người nhận</t>
+          <t>Sổ dự giờ giáo viên có nhận xét và đánh giá tiết dạy</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Lập dự toán kinh phí mua sắm, sửa chữa cơ sở vật chất, bàn ghế phục vụ khai giảng và năm học mới 2026 - 2027</t>
+          <t>Thực hiện kiểm tra đánh giá thường xuyên học sinh theo đúng kế hoạch; chấm bài và vào điểm VnEdu kịp thời</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E64" s="9" t="n">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>Dự toán chi tiết mua sắm, sửa chữa CSVC đầu năm học mới</t>
+          <t>Điểm kiểm tra thường xuyên tháng 9 cập nhật trên VnEdu</t>
         </is>
       </c>
     </row>
@@ -2525,17 +2525,17 @@
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Kiểm kê, vệ sinh, bảo dưỡng toàn bộ thiết bị dạy học, hóa chất, phòng thực hành Lý, Hóa, Sinh trong dịp hè</t>
+          <t>Khảo sát chất lượng đầu năm, phát hiện và lập danh sách học sinh năng khiếu để bồi dưỡng đội tuyển HSG môn phụ trách</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E65" s="9" t="n">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm kê thiết bị dạy học và phòng bộ môn hè 2026</t>
+          <t>Danh sách đội tuyển HSG và Kế hoạch bồi dưỡng HSG</t>
         </is>
       </c>
     </row>
@@ -2559,17 +2559,17 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Tiếp nhận, đóng dấu nghiệp vụ và cấp phát SGK mới, tài liệu hướng dẫn giảng dạy cho GV và HS chuẩn bị năm học mới</t>
+          <t>Lập danh sách học sinh học lực yếu kém đầu năm học để xây dựng phương án dạy phụ đạo, kèm cặp nâng cao chất lượng</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="E66" s="9" t="n">
@@ -2583,27 +2583,27 @@
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
-          <t>Sổ đăng ký cá biệt và danh sách cấp phát sách giáo khoa mới</t>
+          <t>Kế hoạch phụ đạo học sinh có kết quả khảo sát đầu năm thấp</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Bảo dưỡng phòng máy tính tin học, kiểm tra tài khoản VnEdu, CSDL ngành, học bạ số và chữ ký số chuẩn bị năm học mới</t>
+          <t>Đăng ký tên đề tài Sáng kiến kinh nghiệm hoặc Đề tài nghiên cứu khoa học sư phạm ứng dụng năm học 2026 - 2027</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E67" s="9" t="n">
@@ -2617,27 +2617,27 @@
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>Biên bản kiểm tra hệ thống CNTT và phần mềm quản lý trường học</t>
+          <t>Phiếu đăng ký đề tài SKKN năm học 2026-2027 nộp Tổ chuyên môn</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Lập hồ sơ rút dự toán thanh toán tiền lương, phụ cấp tháng 9/2026 và trích nộp BHXH, BHYT, KPCĐ đúng thời hạn</t>
+          <t>Xây dựng Kế hoạch tự bồi dưỡng thường xuyên cá nhân năm học 2026 - 2027 theo quy định của Bộ và Sở GD&amp;ĐT</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="E68" s="9" t="n">
@@ -2651,27 +2651,27 @@
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Bảng thanh toán lương tháng 9/2026 và chứng từ nộp bảo hiểm xã hội</t>
+          <t>Bản kế hoạch tự học, bồi dưỡng thường xuyên năm học 2026-2027</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra thể thức, lấy số, phát hành các quyết định phân công chuyên môn, kế hoạch khai giảng và văn bản đầu năm học</t>
+          <t>Rút dự toán thanh toán tiền lương, các khoản phụ cấp tháng 5/2026 và kinh phí hoạt động chuyên môn cuối năm học đúng quy định</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="E69" s="9" t="n">
@@ -2685,27 +2685,27 @@
       </c>
       <c r="H69" s="10" t="inlineStr">
         <is>
-          <t>Sổ theo dõi văn bản đi tháng 9/2026</t>
+          <t>Giấy rút dự toán ngân sách và bảng thanh toán lương tháng 5/2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Quản lý con dấu, chứng thư số; thực hiện đóng dấu giấy xác nhận học sinh, chứng chỉ cho học sinh đầu năm đúng quy định</t>
+          <t>Tiếp nhận, xử lý và phân phối kịp thời văn bản chỉ đạo của Sở GD&amp;ĐT về thi tốt nghiệp, tuyển sinh 10 và tổng kết năm học</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="E70" s="9" t="n">
@@ -2719,27 +2719,27 @@
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>Sổ cấp giấy xác nhận học sinh năm học 2026-2027</t>
+          <t>Sổ theo dõi văn bản đến tháng 5/2026 trên iOffice</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Mở sổ quỹ tiền mặt năm học 2026 - 2027, ghi chép thu chi quỹ tháng 9 chính xác, thực hiện kiểm kê quỹ cuối tháng</t>
+          <t>Kiểm tra, đóng dấu xác nhận và ký số học bạ số, phiếu điểm cho học sinh lớp 12 phục vụ hồ sơ đăng ký dự thi tốt nghiệp và xét tuyển ĐH</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="E71" s="9" t="n">
@@ -2753,27 +2753,27 @@
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>Sổ quỹ tiền mặt tháng 9/2026 có xác nhận của Kế toán và Hiệu trưởng</t>
+          <t>Sổ theo dõi đóng dấu học bạ và chứng nhận học sinh khối 12</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Lập kế hoạch sử dụng phòng học bộ môn và chuẩn bị đầy đủ thiết bị, hóa chất phục vụ các tiết dạy thực hành tháng 9</t>
+          <t>Quản trị kỹ thuật CSDL ngành, kiểm tra đường truyền và hỗ trợ học sinh khối 12 đăng ký dự thi tốt nghiệp trực tuyến trên Cổng dịch vụ công</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="E72" s="9" t="n">
@@ -2787,27 +2787,27 @@
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>Sổ mượn trả thiết bị dạy học tháng 9/2026</t>
+          <t>Nhật ký hỗ trợ kỹ thuật đăng ký dự thi trực tuyến</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Kiểm tra tủ thuốc y tế, bổ sung bông băng thuốc thiết yếu và lập kế hoạch chăm sóc sức khỏe học sinh đầu năm học mới</t>
+          <t>Phục vụ thiết bị âm thanh, ánh sáng, phòng thi cho kỳ kiểm tra cuối kỳ II và Lễ Bế giảng năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="E73" s="9" t="n">
@@ -2821,27 +2821,27 @@
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>Kế hoạch y tế học đường năm học 2026-2027 và danh mục thuốc</t>
+          <t>Sổ theo dõi bàn giao thiết bị phục vụ kỳ thi và sự kiện bế giảng</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Tuyên truyền phòng chống sốt xuất huyết, dịch bệnh mùa thu và phối hợp vận động học sinh tham gia BHYT đạt 100%</t>
+          <t>Lập danh sách, thông báo và thực hiện tiếp nhận thu hồi SGK, tài liệu tham khảo cho mượn năm học 2025 - 2026</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="E74" s="9" t="n">
@@ -2855,44 +2855,927 @@
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo công tác BHYT học sinh tháng 9/2026</t>
+          <t>Sổ theo dõi thu hồi sách giáo khoa mượn của học sinh</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra tủ thuốc y tế, chuẩn bị thuốc sơ cấp cứu phục vụ thi cuối kỳ II, thi thử tốt nghiệp và tuyên truyền phòng chống say nắng, đuối nước</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>15/05/2026</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G75" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H75" s="10" t="inlineStr">
+        <is>
+          <t>Nhật ký chăm sóc sức khỏe học sinh và biên bản kiểm tra y tế</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>Thực hiện thanh toán tiền coi kiểm tra cuối kỳ, khen thưởng học sinh đạt giải năm học 2025 - 2026 và kiểm kê quỹ tiền mặt tháng 5</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H76" s="10" t="inlineStr">
+        <is>
+          <t>Phiếu chi khen thưởng và biên bản kiểm kê quỹ tháng 5/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>Rút dự toán thanh toán tiền lương, các khoản phụ cấp tháng 6/2026 cho cán bộ, giáo viên, nhân viên đúng thời hạn</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F77" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G77" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H77" s="10" t="inlineStr">
+        <is>
+          <t>Giấy rút dự toán ngân sách và bảng thanh toán lương tháng 6/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Tiếp nhận, đăng ký, chuyển giao kịp thời văn bản chỉ đạo của Sở về thi tốt nghiệp THPT và tuyển sinh lớp 10 năm 2026</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H78" s="10" t="inlineStr">
+        <is>
+          <t>Sổ theo dõi văn bản đến tháng 6/2026 trên iOffice</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Chuẩn bị cơ số thuốc, vật tư y tế, phòng y tế phục vụ Điểm thi tốt nghiệp THPT năm 2026 tại trường an toàn</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F79" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H79" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản kiểm tra điều kiện y tế phục vụ kỳ thi tốt nghiệp 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Bảo dưỡng, kiểm tra hệ thống máy vi tính, đường truyền internet, camera giám sát phục vụ thi tốt nghiệp THPT 2026</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H80" s="10" t="inlineStr">
+        <is>
+          <t>Nhật ký kiểm tra thiết bị CNTT phục vụ kỳ thi</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>Thu hồi SGK, tài liệu tham khảo cho mượn năm học 2025 - 2026; xử lý kỹ thuật và sắp xếp lại kho sách thư viện</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>28/06/2026</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F81" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G81" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H81" s="10" t="inlineStr">
+        <is>
+          <t>Sổ theo dõi mượn trả sách thư viện cuối năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B75" s="10" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>Thực hiện đối chiếu số dư tài khoản tiền gửi và hạn mức kinh phí 6 tháng đầu năm 2026 với Kho bạc Nhà nước</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F82" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H82" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản đối chiếu tài khoản với KBNN kỳ 6 tháng đầu năm 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>Lập báo cáo tài chính và báo cáo quyết toán ngân sách nhà nước 6 tháng đầu năm 2026 nộp Sở GD&amp;ĐT</t>
+        </is>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F83" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H83" s="10" t="inlineStr">
+        <is>
+          <t>Báo cáo quyết toán ngân sách 6 tháng đầu năm 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>Tiếp nhận hồ sơ, sao lục học bạ và cấp phát giấy chứng nhận tốt nghiệp tạm thời cho học sinh khối 12 năm 2026</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H84" s="10" t="inlineStr">
+        <is>
+          <t>Sổ cấp phát văn bằng chứng chỉ, giấy chứng nhận tốt nghiệp tạm thời</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>Thu thập, phân loại và lưu trữ toàn bộ hồ sơ thi tốt nghiệp THPT 2026, hồ sơ tuyển sinh 10 và hồ sơ thi đua năm học 2025 - 2026</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>N1_604 - Thu thập hồ sơ tài liệu vào kho lưu trữ, phục vụ khai thác, sử dụng tài liệu lưu trữ</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F85" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H85" s="10" t="inlineStr">
+        <is>
+          <t>Mục lục hồ sơ tài liệu nộp lưu trữ cơ quan đợt hè 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>Chi trả kịp thời tiền làm nhiệm vụ coi thi, chấm thi và tiền phụ cấp làm việc hè cho cán bộ, giáo viên đúng danh sách</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F86" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H86" s="10" t="inlineStr">
+        <is>
+          <t>Bảng thanh toán tiền làm nhiệm vụ thi có chữ ký người nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Lập dự toán kinh phí mua sắm, sửa chữa cơ sở vật chất, bàn ghế phục vụ khai giảng và năm học mới 2026 - 2027</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>N3_695 - Tổng hợp và lập báo cáo tài chính hợp nhất, báo cáo quyết toán năm</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>15/08/2026</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F87" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H87" s="10" t="inlineStr">
+        <is>
+          <t>Dự toán chi tiết mua sắm, sửa chữa CSVC đầu năm học mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm kê, vệ sinh, bảo dưỡng toàn bộ thiết bị dạy học, hóa chất, phòng thực hành Lý, Hóa, Sinh trong dịp hè</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>15/08/2026</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F88" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H88" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản kiểm kê thiết bị dạy học và phòng bộ môn hè 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>Tiếp nhận, đóng dấu nghiệp vụ và cấp phát SGK mới, tài liệu hướng dẫn giảng dạy cho GV và HS chuẩn bị năm học mới</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>N2_1067 - Báo cáo kết quả tổ chức thực hiện ngày Sách và Văn hóa đọc Việt Nam năm 2026</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F89" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G89" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H89" s="10" t="inlineStr">
+        <is>
+          <t>Sổ đăng ký cá biệt và danh sách cấp phát sách giáo khoa mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Bảo dưỡng phòng máy tính tin học, kiểm tra tài khoản VnEdu, CSDL ngành, học bạ số và chữ ký số chuẩn bị năm học mới</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F90" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H90" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản kiểm tra hệ thống CNTT và phần mềm quản lý trường học</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>Lập hồ sơ rút dự toán thanh toán tiền lương, phụ cấp tháng 9/2026 và trích nộp BHXH, BHYT, KPCĐ đúng thời hạn</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>N1_599 - Thực hiện giao dịch kho bạc , ngân hàng</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F91" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H91" s="10" t="inlineStr">
+        <is>
+          <t>Bảng thanh toán lương tháng 9/2026 và chứng từ nộp bảo hiểm xã hội</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra thể thức, lấy số, phát hành các quyết định phân công chuyên môn, kế hoạch khai giảng và văn bản đầu năm học</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>N1_602 - Quản lý và xử lý văn bản đi, đến (Chính quyền + Đảng ủy)</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F92" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H92" s="10" t="inlineStr">
+        <is>
+          <t>Sổ theo dõi văn bản đi tháng 9/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>Quản lý con dấu, chứng thư số; thực hiện đóng dấu giấy xác nhận học sinh, chứng chỉ cho học sinh đầu năm đúng quy định</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>N1_603 - Quản lý và sử dụng con dấu, thiết bị lưu khóa bí mật; thực hiện ký số chuyển thủ tục hành chính trên dịch vụ công</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F93" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H93" s="10" t="inlineStr">
+        <is>
+          <t>Sổ cấp giấy xác nhận học sinh năm học 2026-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Mở sổ quỹ tiền mặt năm học 2026 - 2027, ghi chép thu chi quỹ tháng 9 chính xác, thực hiện kiểm kê quỹ cuối tháng</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>N1_605 - Quản lý thu, chi tiền mặt tại quỹ, Kiêm nhiệm Thủ quỹ cơ quan; thực hiện các giao dịch tại Kho bạc/Ngân hàng</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F94" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H94" s="10" t="inlineStr">
+        <is>
+          <t>Sổ quỹ tiền mặt tháng 9/2026 có xác nhận của Kế toán và Hiệu trưởng</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch sử dụng phòng học bộ môn và chuẩn bị đầy đủ thiết bị, hóa chất phục vụ các tiết dạy thực hành tháng 9</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>N4_182 - Tham mưu Quyết đinh quy định định tiêu chuẩn, định mức về máy móc thiết bị dạy học</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F95" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H95" s="10" t="inlineStr">
+        <is>
+          <t>Sổ mượn trả thiết bị dạy học tháng 9/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra tủ thuốc y tế, bổ sung bông băng thuốc thiết yếu và lập kế hoạch chăm sóc sức khỏe học sinh đầu năm học mới</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F96" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H96" s="10" t="inlineStr">
+        <is>
+          <t>Kế hoạch y tế học đường năm học 2026-2027 và danh mục thuốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Tuyên truyền phòng chống sốt xuất huyết, dịch bệnh mùa thu và phối hợp vận động học sinh tham gia BHYT đạt 100%</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>N2_1066 - Báo cáo công tác xây dựng giáo dục môi trường an toàn lành mạnh và phòng chống bạo lực học đường</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F97" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H97" s="10" t="inlineStr">
+        <is>
+          <t>Báo cáo công tác BHYT học sinh tháng 9/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>Đưa tin bài, hình ảnh Lễ Khai giảng năm học 2026 - 2027 lên website trường; sao lưu an toàn CSDL tháng 9/2026</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
         <is>
           <t>N2_1085 - Triển khai cảnh báo các lỗ hổng bảo mật, an toàn thông tin theo hướng dẫn của cơ quan chuyên môn</t>
         </is>
       </c>
-      <c r="D75" s="9" t="inlineStr">
+      <c r="D98" s="9" t="inlineStr">
         <is>
           <t>25/09/2026</t>
         </is>
       </c>
-      <c r="E75" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="F75" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="G75" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="H75" s="10" t="inlineStr">
+      <c r="E98" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F98" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
         <is>
           <t>Link bài viết trên website trường và file nhật ký sao lưu hệ thống</t>
         </is>
       </c>
     </row>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:L2"/>

</xml_diff>